<commit_message>
vault backup: 2026-07-03 17:12:44
</commit_message>
<xml_diff>
--- a/Daily-Task-List/Knowledge_Base/WTO-IOTC/教学大纲/相关书籍/书籍链接.xlsx
+++ b/Daily-Task-List/Knowledge_Base/WTO-IOTC/教学大纲/相关书籍/书籍链接.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\1_Learning_Record\1_Typora\My-NoteBook\Daily-Task-List\Knowledge_Base\WTO-IOTC\教学大纲\《国际渔业法》\相关书籍\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\1_Learning_Record\1_Typora\My-NoteBook\Daily-Task-List\Knowledge_Base\WTO-IOTC\教学大纲\相关书籍\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2AA74925-4267-4273-B111-EB846E01B8E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82CBAAD6-7CB9-4137-90A1-4C4BF8767FEE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="29">
   <si>
     <t>书籍</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -99,10 +99,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>WTO读者指南</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>The WTO Agreement on Fisheries Subsidies: A Reader’s Guide</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -116,6 +112,34 @@
   </si>
   <si>
     <t>华敬炘：《渔业法学通论》（上下册） 中国海洋大学出版社，2017。ISBN（下册）：978-7-5670-1448-0</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>渔业法规与渔政管理，中国农业出版社，2010年</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>适用课程</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>《国际渔业法》</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>《国际渔业管理与法规》</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>《国际渔业法》、《国际渔业管理与法规》</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://openknowledge.fao.org/server/api/core/bitstreams/4882e6ba-6715-4510-be11-699989cc8dc1/content</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>A fishery manager's guidebook - Second edition</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -482,144 +506,204 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="102.5" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="102.5" customWidth="1"/>
-    <col min="3" max="3" width="11" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="102.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="102.5" customWidth="1"/>
+    <col min="4" max="4" width="11" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="121.08203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C1" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="D1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="E1" s="4" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:5" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>12</v>
       </c>
       <c r="B2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C2" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="D2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="E2" s="2" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:5" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>11</v>
       </c>
       <c r="B3" t="s">
+        <v>26</v>
+      </c>
+      <c r="C3" t="s">
         <v>8</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="D3" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="E3" s="2" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:5" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
+        <v>22</v>
+      </c>
+      <c r="B4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E4" s="2"/>
+    </row>
+    <row r="5" spans="1:5" ht="16.5" x14ac:dyDescent="0.45">
+      <c r="A5" t="s">
         <v>10</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B5" t="s">
+        <v>24</v>
+      </c>
+      <c r="C5" t="s">
         <v>9</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="D5" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="E5" s="2" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="16.5" x14ac:dyDescent="0.45">
-      <c r="A5" t="s">
+    <row r="6" spans="1:5" ht="16.5" x14ac:dyDescent="0.45">
+      <c r="A6" t="s">
         <v>14</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B6" t="s">
+        <v>24</v>
+      </c>
+      <c r="C6" t="s">
         <v>9</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="D6" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="E6" s="2" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="16.5" x14ac:dyDescent="0.45">
-      <c r="A6" t="s">
+    <row r="7" spans="1:5" ht="16.5" x14ac:dyDescent="0.45">
+      <c r="A7" t="s">
         <v>16</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B7" t="s">
+        <v>24</v>
+      </c>
+      <c r="C7" t="s">
         <v>9</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="D7" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D6" s="2" t="s">
+      <c r="E7" s="2" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="16.5" x14ac:dyDescent="0.45">
-      <c r="A7" t="s">
+    <row r="8" spans="1:5" ht="16.5" x14ac:dyDescent="0.45">
+      <c r="A8" t="s">
+        <v>18</v>
+      </c>
+      <c r="B8" t="s">
+        <v>24</v>
+      </c>
+      <c r="C8" t="s">
+        <v>9</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="16.5" x14ac:dyDescent="0.45">
+      <c r="A9" t="s">
+        <v>20</v>
+      </c>
+      <c r="B9" t="s">
+        <v>24</v>
+      </c>
+      <c r="C9" t="s">
+        <v>9</v>
+      </c>
+      <c r="D9" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="B7" t="s">
-        <v>18</v>
-      </c>
-      <c r="C7" s="1" t="s">
+    </row>
+    <row r="10" spans="1:5" ht="16.5" x14ac:dyDescent="0.45">
+      <c r="A10" t="s">
+        <v>21</v>
+      </c>
+      <c r="B10" t="s">
+        <v>24</v>
+      </c>
+      <c r="C10" t="s">
+        <v>9</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="16.5" x14ac:dyDescent="0.45">
+      <c r="A11" t="s">
+        <v>28</v>
+      </c>
+      <c r="B11" t="s">
+        <v>25</v>
+      </c>
+      <c r="C11" t="s">
+        <v>9</v>
+      </c>
+      <c r="D11" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D7" s="2" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" ht="16.5" x14ac:dyDescent="0.45">
-      <c r="A8" t="s">
-        <v>21</v>
-      </c>
-      <c r="B8" t="s">
-        <v>9</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" ht="16.5" x14ac:dyDescent="0.45">
-      <c r="A9" t="s">
-        <v>22</v>
-      </c>
-      <c r="B9" t="s">
-        <v>9</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>20</v>
+      <c r="E11" s="2" t="s">
+        <v>27</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <hyperlinks>
-    <hyperlink ref="D2" r:id="rId1" xr:uid="{7065177A-F66B-4FC1-9BB0-215465FF10E4}"/>
-    <hyperlink ref="D3" r:id="rId2" xr:uid="{A974B0D1-53B1-4245-A623-8135AC57E345}"/>
-    <hyperlink ref="D4" r:id="rId3" xr:uid="{8581CF74-BF57-4587-804A-6DF07BC4062E}"/>
-    <hyperlink ref="D5" r:id="rId4" xr:uid="{DEF82C2E-8F9F-4EBA-9084-452EC88D4C9E}"/>
-    <hyperlink ref="D6" r:id="rId5" xr:uid="{D0418401-7BDD-4F85-9E6C-6EF4716DE911}"/>
-    <hyperlink ref="D7" r:id="rId6" xr:uid="{67ADFC54-6F2C-4FD0-B417-140F6044E390}"/>
+    <hyperlink ref="E2" r:id="rId1" xr:uid="{7065177A-F66B-4FC1-9BB0-215465FF10E4}"/>
+    <hyperlink ref="E3" r:id="rId2" xr:uid="{A974B0D1-53B1-4245-A623-8135AC57E345}"/>
+    <hyperlink ref="E5" r:id="rId3" xr:uid="{8581CF74-BF57-4587-804A-6DF07BC4062E}"/>
+    <hyperlink ref="E6" r:id="rId4" xr:uid="{DEF82C2E-8F9F-4EBA-9084-452EC88D4C9E}"/>
+    <hyperlink ref="E7" r:id="rId5" xr:uid="{D0418401-7BDD-4F85-9E6C-6EF4716DE911}"/>
+    <hyperlink ref="E8" r:id="rId6" xr:uid="{67ADFC54-6F2C-4FD0-B417-140F6044E390}"/>
+    <hyperlink ref="E11" r:id="rId7" xr:uid="{9D31A334-32CB-4B88-90F3-6BF024594D2F}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
vault backup: 2026-07-03 17:14:36
</commit_message>
<xml_diff>
--- a/Daily-Task-List/Knowledge_Base/WTO-IOTC/教学大纲/相关书籍/书籍链接.xlsx
+++ b/Daily-Task-List/Knowledge_Base/WTO-IOTC/教学大纲/相关书籍/书籍链接.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\1_Learning_Record\1_Typora\My-NoteBook\Daily-Task-List\Knowledge_Base\WTO-IOTC\教学大纲\相关书籍\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82CBAAD6-7CB9-4137-90A1-4C4BF8767FEE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F9E0699-F676-419A-B6FB-021D71580C6A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="30">
   <si>
     <t>书籍</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -140,6 +140,10 @@
   </si>
   <si>
     <t>A fishery manager's guidebook - Second edition</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>国际渔业条约和文件选编，海洋出版社，2014</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -506,7 +510,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="102.5" bestFit="1" customWidth="1"/>
@@ -692,6 +696,20 @@
       </c>
       <c r="E11" s="2" t="s">
         <v>27</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" ht="16.5" x14ac:dyDescent="0.45">
+      <c r="A12" t="s">
+        <v>29</v>
+      </c>
+      <c r="B12" t="s">
+        <v>25</v>
+      </c>
+      <c r="C12" t="s">
+        <v>9</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>19</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
vault backup: 2026-07-03 17:17:15
</commit_message>
<xml_diff>
--- a/Daily-Task-List/Knowledge_Base/WTO-IOTC/教学大纲/相关书籍/书籍链接.xlsx
+++ b/Daily-Task-List/Knowledge_Base/WTO-IOTC/教学大纲/相关书籍/书籍链接.xlsx
@@ -8,13 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\1_Learning_Record\1_Typora\My-NoteBook\Daily-Task-List\Knowledge_Base\WTO-IOTC\教学大纲\相关书籍\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F9E0699-F676-419A-B6FB-021D71580C6A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC8B7F30-0F69-421F-9CB4-123431614C59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="参考教材与阅读书目" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">参考教材与阅读书目!$B$1:$D$12</definedName>
+  </definedNames>
   <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -713,6 +716,7 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="B1:D12" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <phoneticPr fontId="1" type="noConversion"/>
   <hyperlinks>
     <hyperlink ref="E2" r:id="rId1" xr:uid="{7065177A-F66B-4FC1-9BB0-215465FF10E4}"/>

</xml_diff>

<commit_message>
vault backup: 2026-07-03 19:33:28
</commit_message>
<xml_diff>
--- a/Daily-Task-List/Knowledge_Base/WTO-IOTC/教学大纲/相关书籍/书籍链接.xlsx
+++ b/Daily-Task-List/Knowledge_Base/WTO-IOTC/教学大纲/相关书籍/书籍链接.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\1_Learning_Record\1_Typora\My-NoteBook\Daily-Task-List\Knowledge_Base\WTO-IOTC\教学大纲\相关书籍\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC8B7F30-0F69-421F-9CB4-123431614C59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8510149A-5002-46FF-A8B1-024F1E7DD825}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="43">
   <si>
     <t>书籍</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -148,6 +148,57 @@
   <si>
     <t>国际渔业条约和文件选编，海洋出版社，2014</t>
     <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://api.pageplace.de/preview/DT0400.9780192524645_A35502731/preview-9780192524645_A35502731.pdf</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>《国际渔业组织与全球治理》</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>The Oxford Handbook on the United Nations (2nd edn.)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://api.pageplace.de/preview/DT0400.9781351216210_A38998494/preview-9781351216210_A38998494.pdf</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Marine Policy: An Introduction to Governance and International Law of the Oceans (2nd edn.). Routledge: 2019.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://scholarlycommons.law.cwsl.edu/cgi/viewcontent.cgi?article=1337&amp;context=cwilj</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>学术文章</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Mack, J. R. (1995). International fisheries management: how the UN Conference on Straddling and Highly Migratory Fish Stocks changes the law of fishing on the high seas. Cal. W. Int'l LJ, 26, 313.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://s3-us-west-2.amazonaws.com/legacy.seaaroundus/doc/Researcher+Publications/dpauly/PDF/2010/JournalArticles/Cullis-Pauly-Failing-high-seas-global-evaluation(2010).pdf</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Cullis-Suzuki, S., &amp; Pauly, D. (2010). Failing the high seas: a global evaluation of regional fisheries management organizations. Marine Policy, 34(5), 1036-1042.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Allison, E. H., &amp; Ellis, F. (2001). The livelihoods approach and management of small-scale fisheries. Marine policy, 25(5), 377-388.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Petrossian, G. A. (2015). Preventing illegal, unreported and unregulated (IUU) fishing: A situational approach. Biological Conservation, 189, 39-48.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>De Santo, E. M. (2018). Implementation challenges of area-based management tools (ABMTs) for biodiversity beyond national jurisdiction (BBNJ). Marine Policy, 97, 34-43.</t>
   </si>
 </sst>
 </file>
@@ -513,7 +564,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="102.5" bestFit="1" customWidth="1"/>
@@ -715,6 +766,116 @@
         <v>19</v>
       </c>
     </row>
+    <row r="13" spans="1:5" ht="16.5" x14ac:dyDescent="0.45">
+      <c r="A13" t="s">
+        <v>32</v>
+      </c>
+      <c r="B13" t="s">
+        <v>31</v>
+      </c>
+      <c r="C13" t="s">
+        <v>9</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" ht="16.5" x14ac:dyDescent="0.45">
+      <c r="A14" t="s">
+        <v>34</v>
+      </c>
+      <c r="B14" t="s">
+        <v>31</v>
+      </c>
+      <c r="C14" t="s">
+        <v>9</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" ht="16.5" x14ac:dyDescent="0.45">
+      <c r="A15" t="s">
+        <v>37</v>
+      </c>
+      <c r="B15" t="s">
+        <v>31</v>
+      </c>
+      <c r="C15" t="s">
+        <v>36</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" ht="16.5" x14ac:dyDescent="0.45">
+      <c r="A16" t="s">
+        <v>39</v>
+      </c>
+      <c r="B16" t="s">
+        <v>31</v>
+      </c>
+      <c r="C16" t="s">
+        <v>36</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" ht="16.5" x14ac:dyDescent="0.45">
+      <c r="A17" t="s">
+        <v>40</v>
+      </c>
+      <c r="B17" t="s">
+        <v>31</v>
+      </c>
+      <c r="C17" t="s">
+        <v>36</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" ht="16.5" x14ac:dyDescent="0.45">
+      <c r="A18" t="s">
+        <v>41</v>
+      </c>
+      <c r="B18" t="s">
+        <v>31</v>
+      </c>
+      <c r="C18" t="s">
+        <v>36</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" ht="16.5" x14ac:dyDescent="0.45">
+      <c r="A19" t="s">
+        <v>42</v>
+      </c>
+      <c r="B19" t="s">
+        <v>31</v>
+      </c>
+      <c r="C19" t="s">
+        <v>36</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="B1:D12" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <phoneticPr fontId="1" type="noConversion"/>
@@ -726,7 +887,12 @@
     <hyperlink ref="E7" r:id="rId5" xr:uid="{D0418401-7BDD-4F85-9E6C-6EF4716DE911}"/>
     <hyperlink ref="E8" r:id="rId6" xr:uid="{67ADFC54-6F2C-4FD0-B417-140F6044E390}"/>
     <hyperlink ref="E11" r:id="rId7" xr:uid="{9D31A334-32CB-4B88-90F3-6BF024594D2F}"/>
+    <hyperlink ref="E13" r:id="rId8" xr:uid="{0C95729C-3524-4A07-8544-5A0B96CCFFC1}"/>
+    <hyperlink ref="E14" r:id="rId9" xr:uid="{F9952F00-B99B-46A2-ABE4-59D3ADB8BA7F}"/>
+    <hyperlink ref="E15" r:id="rId10" xr:uid="{0BD039C3-79AB-4144-92E1-9486B47DF432}"/>
+    <hyperlink ref="E16" r:id="rId11" xr:uid="{DA44A439-CB79-4558-AA1A-30362E6E2C16}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId12"/>
 </worksheet>
 </file>
</xml_diff>